<commit_message>
update test group booking
</commit_message>
<xml_diff>
--- a/test_data/swing_ios_test_data.xlsx
+++ b/test_data/swing_ios_test_data.xlsx
@@ -8603,7 +8603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8632,7 +8632,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One row per player of a tee time booking, matched on TC_ID. Player No 1 with Add Method host is the booker. Up to 3 players.</t>
+          <t>One row per player of a tee time booking, matched on TC_ID. Player No 1 with Add Method host is the booker. Up to 3 players. Group booking: each invited player logs in with Phone Number on the simulator in Device UDID, one row per device, each with its own WDA Port.</t>
         </is>
       </c>
     </row>
@@ -8710,6 +8710,36 @@
       <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Country Name</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Verification Method</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Device UDID</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>Device Name</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Platform Version</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>WDA Port</t>
         </is>
       </c>
     </row>
@@ -9186,10 +9216,43 @@
           <t>Automation Expired</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>812312312</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>[Testing] Rainbow Morning Promo</t>
         </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>3359EB72-BD7D-4124-98C2-E76DA363D637</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>8101</v>
       </c>
     </row>
     <row r="17">
@@ -9221,6 +9284,11 @@
           <t>Automation Expired</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>812312312</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>[Testing] Rainbow Automation Redeemed</t>
@@ -9239,6 +9307,34 @@
       <c r="N17" t="n">
         <v>1</v>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>3359EB72-BD7D-4124-98C2-E76DA363D637</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>8101</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9269,10 +9365,43 @@
           <t>Automation Expired</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>812312312</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>[Testing] Rainbow Morning Promo</t>
         </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>3359EB72-BD7D-4124-98C2-E76DA363D637</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>8101</v>
       </c>
     </row>
     <row r="19">
@@ -9304,10 +9433,43 @@
           <t>Automation Expired</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>812312312</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>[Testing] Rainbow Morning Promo</t>
         </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>3359EB72-BD7D-4124-98C2-E76DA363D637</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>8101</v>
       </c>
     </row>
     <row r="20">
@@ -9339,10 +9501,43 @@
           <t>Automation Expired</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>812312312</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
           <t>[Testing] Rainbow Morning Promo</t>
         </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>3359EB72-BD7D-4124-98C2-E76DA363D637</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>8101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update for regresss existing
</commit_message>
<xml_diff>
--- a/test_data/swing_ios_test_data.xlsx
+++ b/test_data/swing_ios_test_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="29900" windowHeight="16140" tabRatio="600" firstSheet="1" activeTab="7" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="29900" windowHeight="16140" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,11 +21,11 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Login'!$A$4:$N$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Onboarding'!$A$4:$Y$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Driving Range'!$A$4:$U$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tee Time'!$A$4:$U$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Players'!$A$4:$O$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Driving Range'!$A$4:$U$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tee Time'!$A$4:$U$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Players'!$A$4:$O$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Swing Credits'!$A$4:$K$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Event'!$A$4:$P$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Event'!$A$4:$P$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Add_ons'!$A$4:$C$12</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -762,7 +762,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -819,6 +819,7 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1629,7 +1630,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -1639,7 +1640,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Event Packages - Test Data</t>
@@ -1653,7 +1654,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC_ID</t>
@@ -1753,7 +1754,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -1764,7 +1765,7 @@
     <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20.4" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Player Details - Test Data</t>
@@ -1778,7 +1779,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="17" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TC_ID</t>
@@ -3352,7 +3353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:Z45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3498,6 +3499,31 @@
           <t>Payment Method</t>
         </is>
       </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>Payment Type</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>Card Number</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>Card Expiry</t>
+        </is>
+      </c>
+      <c r="Y4" s="3" t="inlineStr">
+        <is>
+          <t>Card CVV</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
+        <is>
+          <t>Card OTP</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -5743,8 +5769,1428 @@
       <c r="T31" s="4" t="n"/>
       <c r="U31" s="4" t="n"/>
     </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_001</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Credit card</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R32" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S32" s="4" t="n"/>
+      <c r="T32" s="4" t="n"/>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="W32" s="24" t="inlineStr">
+        <is>
+          <t>4000000000002503</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>12/30</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="Z32" s="4" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_002</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with QRIS</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="Q33" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R33" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S33" s="4" t="n"/>
+      <c r="T33" s="4" t="n"/>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>QRIS</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>QRIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_003</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with OVO</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R34" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S34" s="4" t="n"/>
+      <c r="T34" s="4" t="n"/>
+      <c r="U34" s="4" t="inlineStr">
+        <is>
+          <t>OVO</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="34" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_004</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Shopee Pay</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R35" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S35" s="4" t="n"/>
+      <c r="T35" s="4" t="n"/>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>Shopee Pay</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_005</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with LinkAja</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="P36" s="4" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R36" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S36" s="4" t="n"/>
+      <c r="T36" s="4" t="n"/>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>LinkAja</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_006</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with DANA</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R37" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S37" s="4" t="n"/>
+      <c r="T37" s="4" t="n"/>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>DANA</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="34" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_007</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank BJB</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R38" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S38" s="4" t="n"/>
+      <c r="T38" s="4" t="n"/>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>Bank BJB</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_008</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank CIMB</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="n"/>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R39" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S39" s="4" t="n"/>
+      <c r="T39" s="4" t="n"/>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>Bank CIMB</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="34" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_009</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank Mandiri</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="P40" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R40" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S40" s="4" t="n"/>
+      <c r="T40" s="4" t="n"/>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>Bank Mandiri</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="34" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_010</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank BRI</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R41" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S41" s="4" t="n"/>
+      <c r="T41" s="4" t="n"/>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>Bank BRI</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="34" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_011</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank Permata</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="P42" s="4" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="Q42" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R42" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S42" s="4" t="n"/>
+      <c r="T42" s="4" t="n"/>
+      <c r="U42" s="4" t="inlineStr">
+        <is>
+          <t>Bank Permata</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_012</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank BNI</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="n"/>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="P43" s="4" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R43" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S43" s="4" t="n"/>
+      <c r="T43" s="4" t="n"/>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>Bank BNI</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="34" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_013</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank BSI</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="n"/>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="P44" s="4" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="Q44" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R44" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S44" s="4" t="n"/>
+      <c r="T44" s="4" t="n"/>
+      <c r="U44" s="4" t="inlineStr">
+        <is>
+          <t>Bank BSI</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="34" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>DR_REGRESS_GSA_014</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Booking Driving Range Indonesia paid with Bank Sahabat Sampoerna</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Driving Range</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>Albatross Driving Range</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>15 October 2026</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr">
+        <is>
+          <t>Regular</t>
+        </is>
+      </c>
+      <c r="R45" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S45" s="4" t="n"/>
+      <c r="T45" s="4" t="n"/>
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>Bank Sahabat Sampoerna</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:U31"/>
+  <autoFilter ref="A4:U45"/>
   <dataValidations count="2">
     <dataValidation sqref="D5:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"UI,Positive,Negative,E2E"</formula1>
@@ -5763,7 +7209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y31"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5929,6 +7375,31 @@
           <t>Player Name</t>
         </is>
       </c>
+      <c r="Z4" s="3" t="inlineStr">
+        <is>
+          <t>Payment Type</t>
+        </is>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>Card Number</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>Card Expiry</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>Card CVV</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>Card OTP</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -7988,7 +9459,7 @@
       </c>
       <c r="U26" s="4" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="34" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>TT_GB_001</t>
@@ -8107,7 +9578,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="34" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>TT_GB_002</t>
@@ -8226,7 +9697,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="34" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>TT_GB_003</t>
@@ -8345,7 +9816,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="34" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>TT_GB_004</t>
@@ -8464,7 +9935,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="34" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
           <t>TT_GB_005</t>
@@ -8583,8 +10054,1428 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_001</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Credit card</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N32" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P32" s="21" t="inlineStr">
+        <is>
+          <t>06:30 - 07:00</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R32" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S32" s="4" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="T32" s="4" t="n"/>
+      <c r="U32" s="4" t="n"/>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>4000000000001091</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>12/30</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="AD32" s="4" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_002</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with QRIS</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="n"/>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N33" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P33" s="21" t="inlineStr">
+        <is>
+          <t>07:00 - 07:30</t>
+        </is>
+      </c>
+      <c r="Q33" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R33" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S33" s="4" t="inlineStr">
+        <is>
+          <t>QRIS</t>
+        </is>
+      </c>
+      <c r="T33" s="4" t="n"/>
+      <c r="U33" s="4" t="n"/>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>QRIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_003</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with OVO</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N34" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P34" s="21" t="inlineStr">
+        <is>
+          <t>07:30 - 08:00</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R34" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>OVO</t>
+        </is>
+      </c>
+      <c r="T34" s="4" t="n"/>
+      <c r="U34" s="4" t="n"/>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="34" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_004</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Shopee Pay</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N35" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P35" s="21" t="inlineStr">
+        <is>
+          <t>08:00 - 08:30</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R35" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>Shopee Pay</t>
+        </is>
+      </c>
+      <c r="T35" s="4" t="n"/>
+      <c r="U35" s="4" t="n"/>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_005</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with LinkAja</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N36" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P36" s="21" t="inlineStr">
+        <is>
+          <t>08:30 - 09:00</t>
+        </is>
+      </c>
+      <c r="Q36" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R36" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S36" s="4" t="inlineStr">
+        <is>
+          <t>LinkAja</t>
+        </is>
+      </c>
+      <c r="T36" s="4" t="n"/>
+      <c r="U36" s="4" t="n"/>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_006</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with DANA</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N37" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P37" s="21" t="inlineStr">
+        <is>
+          <t>09:00 - 09:30</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R37" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S37" s="4" t="inlineStr">
+        <is>
+          <t>DANA</t>
+        </is>
+      </c>
+      <c r="T37" s="4" t="n"/>
+      <c r="U37" s="4" t="n"/>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>E-wallet</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="34" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_007</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank BJB</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N38" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P38" s="21" t="inlineStr">
+        <is>
+          <t>09:30 - 10:00</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R38" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S38" s="4" t="inlineStr">
+        <is>
+          <t>Bank BJB</t>
+        </is>
+      </c>
+      <c r="T38" s="4" t="n"/>
+      <c r="U38" s="4" t="n"/>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_008</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank CIMB</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="n"/>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N39" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P39" s="21" t="inlineStr">
+        <is>
+          <t>10:00 - 10:30</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R39" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S39" s="4" t="inlineStr">
+        <is>
+          <t>Bank CIMB</t>
+        </is>
+      </c>
+      <c r="T39" s="4" t="n"/>
+      <c r="U39" s="4" t="n"/>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="34" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_009</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank Mandiri</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="n"/>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N40" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P40" s="21" t="inlineStr">
+        <is>
+          <t>10:30 - 11:00</t>
+        </is>
+      </c>
+      <c r="Q40" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R40" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S40" s="4" t="inlineStr">
+        <is>
+          <t>Bank Mandiri</t>
+        </is>
+      </c>
+      <c r="T40" s="4" t="n"/>
+      <c r="U40" s="4" t="n"/>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="34" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_010</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank BRI</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="n"/>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N41" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P41" s="21" t="inlineStr">
+        <is>
+          <t>11:00 - 11:30</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R41" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S41" s="4" t="inlineStr">
+        <is>
+          <t>Bank BRI</t>
+        </is>
+      </c>
+      <c r="T41" s="4" t="n"/>
+      <c r="U41" s="4" t="n"/>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="34" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_011</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank Permata</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N42" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P42" s="21" t="inlineStr">
+        <is>
+          <t>11:30 - 12:00</t>
+        </is>
+      </c>
+      <c r="Q42" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R42" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S42" s="4" t="inlineStr">
+        <is>
+          <t>Bank Permata</t>
+        </is>
+      </c>
+      <c r="T42" s="4" t="n"/>
+      <c r="U42" s="4" t="n"/>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_012</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank BNI</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="n"/>
+      <c r="J43" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N43" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P43" s="21" t="inlineStr">
+        <is>
+          <t>12:00 - 12:30</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R43" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S43" s="4" t="inlineStr">
+        <is>
+          <t>Bank BNI</t>
+        </is>
+      </c>
+      <c r="T43" s="4" t="n"/>
+      <c r="U43" s="4" t="n"/>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="34" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_013</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank BSI</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="n"/>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N44" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>Day Session</t>
+        </is>
+      </c>
+      <c r="P44" s="21" t="inlineStr">
+        <is>
+          <t>12:30 - 13:00</t>
+        </is>
+      </c>
+      <c r="Q44" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R44" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S44" s="4" t="inlineStr">
+        <is>
+          <t>Bank BSI</t>
+        </is>
+      </c>
+      <c r="T44" s="4" t="n"/>
+      <c r="U44" s="4" t="n"/>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="34" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>TT_REGRESS_GSA_014</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Book a standard tee time Indonesia, host only, paid with Bank Sahabat Sampoerna</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Tee Time</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>E2E</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>812312314</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="11" t="inlineStr">
+        <is>
+          <t>Automation Swing Pass</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>swing-pass</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>Rainbow Hills Golf</t>
+        </is>
+      </c>
+      <c r="N45" s="21" t="inlineStr">
+        <is>
+          <t>16 October 2026</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>Night Session</t>
+        </is>
+      </c>
+      <c r="P45" s="21" t="inlineStr">
+        <is>
+          <t>13:00 - 13:30</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="R45" s="21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S45" s="4" t="inlineStr">
+        <is>
+          <t>Bank Sahabat Sampoerna</t>
+        </is>
+      </c>
+      <c r="T45" s="4" t="n"/>
+      <c r="U45" s="4" t="n"/>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>Virtual account</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:U26"/>
+  <autoFilter ref="A4:U45"/>
   <dataValidations count="2">
     <dataValidation sqref="D5:D26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"UI,Positive,Negative,E2E"</formula1>
@@ -9451,7 +12342,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O12"/>
+  <autoFilter ref="A4:O20"/>
   <dataValidations count="1">
     <dataValidation sqref="C5 C7 C10 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"host,search,manual"</formula1>
@@ -9804,12 +12695,7 @@
     <col width="56" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="17" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.4" customHeight="1">
@@ -10633,7 +13519,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P12"/>
+  <autoFilter ref="A4:P14"/>
   <dataValidations count="3">
     <dataValidation sqref="D5:D12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Positive,Negative,UI"</formula1>

</xml_diff>